<commit_message>
ChatGPT-style chat (typewriter reveal, Auto toggle, options drawer), Learn lab UI, learning guide, docs and tests
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012muWped4tVffJ87y3fEXZK
</commit_message>
<xml_diff>
--- a/docs/eval/eval_report.xlsx
+++ b/docs/eval/eval_report.xlsx
@@ -760,7 +760,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-30 07:50:40 UTC</t>
+          <t>Generated 2026-10-31 14:59:45 UTC</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18 / 28 ms</t>
+          <t>30 / 43 ms</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>15.3</t>
+          <t>26.4</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>20.5</t>
+          <t>27.4</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>15.8</t>
+          <t>19.9</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>14.8</t>
+          <t>33.9</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>18.7</t>
+          <t>30.4</t>
         </is>
       </c>
     </row>
@@ -1684,12 +1684,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>24.9</t>
+          <t>43.3</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -1726,12 +1726,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>14.8</t>
+          <t>24.1</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>21.4</t>
+          <t>31.7</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -1768,12 +1768,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>16.5</t>
+          <t>22.2</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>22.9</t>
+          <t>37.8</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -1810,12 +1810,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>26.9</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>37.1</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -1852,12 +1852,12 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>16.1</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>22.7</t>
+          <t>42.2</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>27.6</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>24.7</t>
+          <t>40.9</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -2254,7 +2254,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -2604,7 +2604,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -2744,7 +2744,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -2954,7 +2954,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -3059,7 +3059,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -3164,7 +3164,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -3304,7 +3304,7 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -3374,7 +3374,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -3444,7 +3444,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -3479,7 +3479,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -3549,7 +3549,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -3684,17 +3684,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>08342e63af66</t>
+          <t>ba9b0b05a100</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:50:40 UTC</t>
+          <t>2026-10-31 14:59:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3714,12 +3714,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>b3a6c24070a1</t>
+          <t>dabd44ecf45e</t>
         </is>
       </c>
     </row>
@@ -3739,12 +3739,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3dc9560fa396</t>
+          <t>4c5876822788</t>
         </is>
       </c>
     </row>
@@ -3764,12 +3764,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>793a140afb7e</t>
+          <t>a3456d50fc4a</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-30T07:50:39+00:00</t>
+          <t>2026-10-31T14:59:43+00:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">

</xml_diff>